<commit_message>
docs(combat): amplía spec funcional y diseño UI con Modo C y detalle de fórmulas T4.5
Actualiza la documentación del simulador de combate:
- docs/specs/simulador-combate.md: +324 líneas — RN-04 (scoring_mode), RN-05 (n_min/n_max),
  detalle de fórmula de K dinámico y tabla de bonificadores por tipo de tropa
- docs/design/simulador-combate-ui.md: spec visual completo del OptimizerResult Modo C
- docs/specs/oasis-farming.md: parche menor con aclaración de tipos CROP vs RES en Nature drops
- docs/Reporte de ataques.xlsx: datos de referencia actualizados con reportes adicionales
</commit_message>
<xml_diff>
--- a/docs/Reporte de ataques.xlsx
+++ b/docs/Reporte de ataques.xlsx
@@ -53,10 +53,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8.0"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
@@ -80,21 +86,33 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="20" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="20" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="20" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -175,7 +193,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A2:L23" displayName="Atracos" name="Atracos" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A2:L40" displayName="Atracos" name="Atracos" id="1">
   <tableColumns count="12">
     <tableColumn name="ultimo ataque" id="1"/>
     <tableColumn name="Hora check" id="2"/>
@@ -401,407 +419,815 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
     </row>
     <row r="2" ht="22.5" customHeight="1">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="L2" s="3" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
-      <c r="A3" s="3">
+      <c r="A3" s="4">
         <v>0.6513888888888889</v>
       </c>
-      <c r="B3" s="3">
-        <v>0.8472222222222222</v>
-      </c>
-      <c r="C3" s="4">
+      <c r="B3" s="4">
+        <v>0.8472222222222222</v>
+      </c>
+      <c r="C3" s="5">
         <v>10.0</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="5">
         <v>3.0</v>
       </c>
-      <c r="F3" s="4">
+      <c r="F3" s="5">
         <v>5.0</v>
       </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
-      <c r="A4" s="3">
+      <c r="A4" s="4">
         <v>0.6381944444444444</v>
       </c>
-      <c r="B4" s="3">
-        <v>0.8472222222222222</v>
-      </c>
-      <c r="G4" s="4">
+      <c r="B4" s="4">
+        <v>0.8472222222222222</v>
+      </c>
+      <c r="G4" s="5">
         <v>5.0</v>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="5">
         <v>3.0</v>
       </c>
-      <c r="I4" s="4">
+      <c r="I4" s="5">
         <v>1.0</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
-      <c r="A5" s="3">
+      <c r="A5" s="4">
         <v>0.6465277777777778</v>
       </c>
-      <c r="B5" s="3">
-        <v>0.8472222222222222</v>
-      </c>
-      <c r="C5" s="4">
+      <c r="B5" s="4">
+        <v>0.8472222222222222</v>
+      </c>
+      <c r="C5" s="5">
         <v>12.0</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="5">
         <v>10.0</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5" s="5">
         <v>3.0</v>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
-      <c r="A6" s="3">
+      <c r="A6" s="4">
         <v>0.6402777777777777</v>
       </c>
-      <c r="B6" s="3">
-        <v>0.8472222222222222</v>
-      </c>
-      <c r="C6" s="4">
+      <c r="B6" s="4">
+        <v>0.8472222222222222</v>
+      </c>
+      <c r="C6" s="5">
         <v>19.0</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="5">
         <v>9.0</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6" s="5">
         <v>4.0</v>
       </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
-      <c r="A7" s="3">
+      <c r="A7" s="4">
         <v>0.6402777777777777</v>
       </c>
-      <c r="B7" s="3">
-        <v>0.8472222222222222</v>
-      </c>
-      <c r="C7" s="4">
+      <c r="B7" s="4">
+        <v>0.8472222222222222</v>
+      </c>
+      <c r="C7" s="5">
         <v>14.0</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="5">
         <v>11.0</v>
       </c>
-      <c r="G7" s="4">
+      <c r="G7" s="5">
         <v>4.0</v>
       </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="3">
+      <c r="A8" s="4">
         <v>0.6326388888888889</v>
       </c>
-      <c r="B8" s="3">
-        <v>0.8472222222222222</v>
-      </c>
-      <c r="D8" s="4">
+      <c r="B8" s="4">
+        <v>0.8472222222222222</v>
+      </c>
+      <c r="D8" s="5">
         <v>3.0</v>
       </c>
-      <c r="G8" s="4">
+      <c r="G8" s="5">
         <v>9.0</v>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
-      <c r="A9" s="3">
+      <c r="A9" s="4">
         <v>0.6375</v>
       </c>
-      <c r="B9" s="3">
-        <v>0.8472222222222222</v>
-      </c>
-      <c r="C9" s="4">
+      <c r="B9" s="4">
+        <v>0.8472222222222222</v>
+      </c>
+      <c r="C9" s="5">
         <v>6.0</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="5">
         <v>4.0</v>
       </c>
-      <c r="G9" s="4">
+      <c r="G9" s="5">
         <v>2.0</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
-      <c r="A10" s="3">
+      <c r="A10" s="4">
         <v>0.6604166666666667</v>
       </c>
-      <c r="B10" s="3">
-        <v>0.8472222222222222</v>
-      </c>
-      <c r="C10" s="4">
+      <c r="B10" s="4">
+        <v>0.8472222222222222</v>
+      </c>
+      <c r="C10" s="5">
         <v>12.0</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="5">
         <v>4.0</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="5">
         <v>19.0</v>
       </c>
     </row>
     <row r="11" ht="22.5" customHeight="1">
-      <c r="A11" s="3">
+      <c r="A11" s="4">
         <v>0.6638888888888889</v>
       </c>
-      <c r="B11" s="3">
-        <v>0.8472222222222222</v>
-      </c>
-      <c r="C11" s="4">
+      <c r="B11" s="4">
+        <v>0.8472222222222222</v>
+      </c>
+      <c r="C11" s="5">
         <v>6.0</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="5">
         <v>6.0</v>
       </c>
-      <c r="G11" s="4">
+      <c r="G11" s="5">
         <v>3.0</v>
       </c>
     </row>
     <row r="12" ht="22.5" customHeight="1">
-      <c r="A12" s="3">
+      <c r="A12" s="4">
         <v>0.6305555555555555</v>
       </c>
-      <c r="B12" s="3">
-        <v>0.8472222222222222</v>
-      </c>
-      <c r="I12" s="4">
+      <c r="B12" s="4">
+        <v>0.8472222222222222</v>
+      </c>
+      <c r="I12" s="5">
         <v>7.0</v>
       </c>
     </row>
     <row r="13" ht="22.5" customHeight="1">
-      <c r="A13" s="3">
+      <c r="A13" s="4">
         <v>0.6395833333333333</v>
       </c>
-      <c r="B13" s="3">
-        <v>0.8472222222222222</v>
-      </c>
-      <c r="C13" s="4">
+      <c r="B13" s="4">
+        <v>0.8472222222222222</v>
+      </c>
+      <c r="C13" s="5">
         <v>8.0</v>
       </c>
-      <c r="D13" s="4">
+      <c r="D13" s="5">
         <v>6.0</v>
       </c>
-      <c r="G13" s="4">
+      <c r="G13" s="5">
         <v>2.0</v>
       </c>
     </row>
     <row r="14" ht="22.5" customHeight="1">
-      <c r="A14" s="3">
+      <c r="A14" s="4">
         <v>0.6458333333333334</v>
       </c>
-      <c r="B14" s="3">
-        <v>0.8472222222222222</v>
-      </c>
-      <c r="C14" s="4">
+      <c r="B14" s="4">
+        <v>0.8472222222222222</v>
+      </c>
+      <c r="C14" s="5">
         <v>16.0</v>
       </c>
-      <c r="D14" s="4">
+      <c r="D14" s="5">
         <v>8.0</v>
       </c>
-      <c r="E14" s="4">
+      <c r="E14" s="5">
         <v>8.0</v>
       </c>
     </row>
     <row r="15" ht="22.5" customHeight="1">
-      <c r="A15" s="3">
+      <c r="A15" s="4">
         <v>0.6472222222222223</v>
       </c>
-      <c r="B15" s="3">
-        <v>0.8472222222222222</v>
-      </c>
-      <c r="C15" s="4">
+      <c r="B15" s="4">
+        <v>0.8472222222222222</v>
+      </c>
+      <c r="C15" s="5">
         <v>18.0</v>
       </c>
-      <c r="D15" s="4">
+      <c r="D15" s="5">
         <v>8.0</v>
       </c>
-      <c r="E15" s="4">
+      <c r="E15" s="5">
         <v>6.0</v>
       </c>
     </row>
     <row r="16" ht="22.5" customHeight="1">
-      <c r="A16" s="3">
+      <c r="A16" s="4">
         <v>0.6111111111111112</v>
       </c>
-      <c r="B16" s="3">
-        <v>0.8472222222222222</v>
-      </c>
-      <c r="C16" s="4">
+      <c r="B16" s="4">
+        <v>0.8472222222222222</v>
+      </c>
+      <c r="C16" s="5">
         <v>8.0</v>
       </c>
-      <c r="D16" s="4">
+      <c r="D16" s="5">
         <v>4.0</v>
       </c>
-      <c r="G16" s="4">
+      <c r="G16" s="5">
         <v>3.0</v>
       </c>
     </row>
     <row r="17" ht="22.5" customHeight="1">
-      <c r="A17" s="3">
+      <c r="A17" s="4">
         <v>0.6131944444444445</v>
       </c>
-      <c r="B17" s="3">
-        <v>0.8472222222222222</v>
-      </c>
-      <c r="C17" s="4">
+      <c r="B17" s="4">
+        <v>0.8472222222222222</v>
+      </c>
+      <c r="C17" s="5">
         <v>11.0</v>
       </c>
-      <c r="D17" s="4">
+      <c r="D17" s="5">
         <v>6.0</v>
       </c>
-      <c r="E17" s="4">
+      <c r="E17" s="5">
         <v>5.0</v>
       </c>
-      <c r="K17" s="4">
+      <c r="K17" s="5">
         <v>13.0</v>
       </c>
     </row>
     <row r="18" ht="22.5" customHeight="1">
-      <c r="A18" s="3">
+      <c r="A18" s="4">
         <v>0.6555555555555556</v>
       </c>
-      <c r="B18" s="3">
-        <v>0.8472222222222222</v>
-      </c>
-      <c r="C18" s="4">
+      <c r="B18" s="4">
+        <v>0.8472222222222222</v>
+      </c>
+      <c r="C18" s="5">
         <v>20.0</v>
       </c>
-      <c r="D18" s="4">
+      <c r="D18" s="5">
         <v>7.0</v>
       </c>
     </row>
     <row r="19" ht="22.5" customHeight="1">
-      <c r="A19" s="3">
+      <c r="A19" s="4">
         <v>0.6576388888888889</v>
       </c>
-      <c r="B19" s="3">
-        <v>0.8472222222222222</v>
-      </c>
-      <c r="C19" s="4">
+      <c r="B19" s="4">
+        <v>0.8472222222222222</v>
+      </c>
+      <c r="C19" s="5">
         <v>21.0</v>
       </c>
-      <c r="D19" s="4">
+      <c r="D19" s="5">
         <v>15.0</v>
       </c>
-      <c r="E19" s="4">
+      <c r="E19" s="5">
         <v>15.0</v>
       </c>
     </row>
     <row r="20" ht="22.5" customHeight="1">
-      <c r="A20" s="3">
+      <c r="A20" s="4">
         <v>0.6611111111111111</v>
       </c>
-      <c r="B20" s="3">
-        <v>0.8472222222222222</v>
-      </c>
-      <c r="C20" s="4">
+      <c r="B20" s="4">
+        <v>0.8472222222222222</v>
+      </c>
+      <c r="C20" s="5">
         <v>8.0</v>
       </c>
-      <c r="D20" s="4">
+      <c r="D20" s="5">
         <v>4.0</v>
       </c>
-      <c r="E20" s="4">
+      <c r="E20" s="5">
         <v>4.0</v>
       </c>
     </row>
     <row r="21" ht="22.5" customHeight="1">
-      <c r="A21" s="3">
+      <c r="A21" s="4">
         <v>0.6638888888888889</v>
       </c>
-      <c r="B21" s="3">
-        <v>0.8472222222222222</v>
-      </c>
-      <c r="C21" s="4">
+      <c r="B21" s="4">
+        <v>0.8472222222222222</v>
+      </c>
+      <c r="C21" s="5">
         <v>36.0</v>
       </c>
-      <c r="D21" s="4">
+      <c r="D21" s="5">
         <v>15.0</v>
       </c>
-      <c r="E21" s="4">
+      <c r="E21" s="5">
         <v>12.0</v>
       </c>
     </row>
     <row r="22" ht="22.5" customHeight="1">
-      <c r="A22" s="3">
+      <c r="A22" s="4">
         <v>0.6652777777777777</v>
       </c>
-      <c r="B22" s="3">
-        <v>0.8472222222222222</v>
-      </c>
-      <c r="C22" s="4">
+      <c r="B22" s="4">
+        <v>0.8472222222222222</v>
+      </c>
+      <c r="C22" s="5">
         <v>24.0</v>
       </c>
-      <c r="D22" s="4">
+      <c r="D22" s="5">
         <v>12.0</v>
       </c>
-      <c r="E22" s="4">
+      <c r="E22" s="5">
         <v>6.0</v>
       </c>
     </row>
     <row r="23" ht="22.5" customHeight="1">
-      <c r="A23" s="3">
+      <c r="A23" s="4">
         <v>0.7395833333333334</v>
       </c>
-      <c r="B23" s="3">
-        <v>0.8472222222222222</v>
-      </c>
-      <c r="C23" s="4">
+      <c r="B23" s="4">
+        <v>0.8472222222222222</v>
+      </c>
+      <c r="C23" s="5">
         <v>21.0</v>
       </c>
-      <c r="D23" s="4">
+      <c r="D23" s="5">
         <v>8.0</v>
       </c>
-      <c r="E23" s="4">
+      <c r="E23" s="5">
         <v>6.0</v>
       </c>
+    </row>
+    <row r="24" ht="22.5" customHeight="1">
+      <c r="A24" s="6">
+        <v>46170.62847222222</v>
+      </c>
+      <c r="B24" s="6">
+        <v>46171.529861111114</v>
+      </c>
+      <c r="C24" s="7">
+        <v>8.0</v>
+      </c>
+      <c r="D24" s="7">
+        <v>5.0</v>
+      </c>
+      <c r="E24" s="7"/>
+      <c r="F24" s="7">
+        <v>33.0</v>
+      </c>
+      <c r="G24" s="7">
+        <v>2.0</v>
+      </c>
+      <c r="H24" s="8"/>
+      <c r="I24" s="8"/>
+      <c r="J24" s="8"/>
+      <c r="K24" s="8"/>
+      <c r="L24" s="8"/>
+    </row>
+    <row r="25" ht="22.5" customHeight="1">
+      <c r="A25" s="6">
+        <v>46170.62847222222</v>
+      </c>
+      <c r="B25" s="6">
+        <v>46171.80069444444</v>
+      </c>
+      <c r="C25" s="7">
+        <v>6.0</v>
+      </c>
+      <c r="D25" s="7">
+        <v>6.0</v>
+      </c>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="7">
+        <v>2.0</v>
+      </c>
+      <c r="H25" s="8"/>
+      <c r="I25" s="8"/>
+      <c r="J25" s="8"/>
+      <c r="K25" s="8"/>
+      <c r="L25" s="8"/>
+    </row>
+    <row r="26" ht="22.5" customHeight="1">
+      <c r="A26" s="6">
+        <v>46170.631944444445</v>
+      </c>
+      <c r="B26" s="6">
+        <v>46171.0021875</v>
+      </c>
+      <c r="C26" s="7">
+        <v>14.0</v>
+      </c>
+      <c r="D26" s="7">
+        <v>10.0</v>
+      </c>
+      <c r="E26" s="7"/>
+      <c r="F26" s="7"/>
+      <c r="G26" s="7">
+        <v>6.0</v>
+      </c>
+      <c r="H26" s="8"/>
+      <c r="I26" s="8"/>
+      <c r="J26" s="8"/>
+      <c r="K26" s="8"/>
+      <c r="L26" s="8"/>
+    </row>
+    <row r="27" ht="22.5" customHeight="1">
+      <c r="A27" s="6">
+        <v>46171.0021875</v>
+      </c>
+      <c r="B27" s="6">
+        <v>46171.55003472222</v>
+      </c>
+      <c r="C27" s="7">
+        <v>8.0</v>
+      </c>
+      <c r="D27" s="7">
+        <v>5.0</v>
+      </c>
+      <c r="E27" s="7"/>
+      <c r="F27" s="7"/>
+      <c r="G27" s="7">
+        <v>3.0</v>
+      </c>
+      <c r="H27" s="8"/>
+      <c r="I27" s="8"/>
+      <c r="J27" s="8"/>
+      <c r="K27" s="8"/>
+      <c r="L27" s="8"/>
+    </row>
+    <row r="28" ht="22.5" customHeight="1">
+      <c r="A28" s="6">
+        <v>46170.631944444445</v>
+      </c>
+      <c r="B28" s="6">
+        <v>46171.80347222222</v>
+      </c>
+      <c r="C28" s="7">
+        <v>31.0</v>
+      </c>
+      <c r="D28" s="7">
+        <v>17.0</v>
+      </c>
+      <c r="E28" s="7"/>
+      <c r="F28" s="7"/>
+      <c r="G28" s="7">
+        <v>11.0</v>
+      </c>
+      <c r="H28" s="8"/>
+      <c r="I28" s="8"/>
+      <c r="J28" s="8"/>
+      <c r="K28" s="8"/>
+      <c r="L28" s="8"/>
+    </row>
+    <row r="29" ht="22.5" customHeight="1">
+      <c r="A29" s="6">
+        <v>46170.64236111111</v>
+      </c>
+      <c r="B29" s="6">
+        <v>46171.80347222222</v>
+      </c>
+      <c r="C29" s="7">
+        <v>6.0</v>
+      </c>
+      <c r="D29" s="7">
+        <v>5.0</v>
+      </c>
+      <c r="E29" s="7"/>
+      <c r="F29" s="7"/>
+      <c r="G29" s="7">
+        <v>2.0</v>
+      </c>
+      <c r="H29" s="8"/>
+      <c r="I29" s="8"/>
+      <c r="J29" s="8"/>
+      <c r="K29" s="8"/>
+      <c r="L29" s="8"/>
+    </row>
+    <row r="30" ht="22.5" customHeight="1">
+      <c r="A30" s="6">
+        <v>46170.64236111111</v>
+      </c>
+      <c r="B30" s="6">
+        <v>46171.80347222222</v>
+      </c>
+      <c r="C30" s="7">
+        <v>20.0</v>
+      </c>
+      <c r="D30" s="7">
+        <v>12.0</v>
+      </c>
+      <c r="E30" s="7"/>
+      <c r="F30" s="7"/>
+      <c r="G30" s="7">
+        <v>7.0</v>
+      </c>
+      <c r="H30" s="8"/>
+      <c r="I30" s="8"/>
+      <c r="J30" s="8"/>
+      <c r="K30" s="8"/>
+      <c r="L30" s="8"/>
+    </row>
+    <row r="31" ht="22.5" customHeight="1">
+      <c r="A31" s="6">
+        <v>46170.64513888889</v>
+      </c>
+      <c r="B31" s="6">
+        <v>46171.80347222222</v>
+      </c>
+      <c r="C31" s="7">
+        <v>24.0</v>
+      </c>
+      <c r="D31" s="7">
+        <v>15.0</v>
+      </c>
+      <c r="E31" s="7"/>
+      <c r="F31" s="7"/>
+      <c r="G31" s="7">
+        <v>7.0</v>
+      </c>
+      <c r="H31" s="8"/>
+      <c r="I31" s="8"/>
+      <c r="J31" s="8"/>
+      <c r="K31" s="8"/>
+      <c r="L31" s="8"/>
+    </row>
+    <row r="32" ht="22.5" customHeight="1">
+      <c r="A32" s="6">
+        <v>46170.65277777778</v>
+      </c>
+      <c r="B32" s="6">
+        <v>46171.80347222222</v>
+      </c>
+      <c r="C32" s="7">
+        <v>24.0</v>
+      </c>
+      <c r="D32" s="7">
+        <v>8.0</v>
+      </c>
+      <c r="F32" s="7">
+        <v>11.0</v>
+      </c>
+      <c r="G32" s="7"/>
+      <c r="H32" s="8"/>
+      <c r="I32" s="8"/>
+      <c r="J32" s="8"/>
+      <c r="K32" s="8"/>
+      <c r="L32" s="8"/>
+    </row>
+    <row r="33" ht="22.5" customHeight="1">
+      <c r="A33" s="6">
+        <v>46170.87358796296</v>
+      </c>
+      <c r="B33" s="6">
+        <v>46171.432175925926</v>
+      </c>
+      <c r="C33" s="7">
+        <v>9.0</v>
+      </c>
+      <c r="D33" s="7">
+        <v>8.0</v>
+      </c>
+      <c r="F33" s="7">
+        <v>9.0</v>
+      </c>
+      <c r="G33" s="7"/>
+      <c r="H33" s="8"/>
+      <c r="I33" s="8"/>
+      <c r="J33" s="8"/>
+      <c r="K33" s="8"/>
+      <c r="L33" s="8"/>
+    </row>
+    <row r="34" ht="22.5" customHeight="1">
+      <c r="A34" s="6">
+        <v>46170.62986111111</v>
+      </c>
+      <c r="B34" s="6">
+        <v>46171.44421296296</v>
+      </c>
+      <c r="C34" s="7">
+        <v>38.0</v>
+      </c>
+      <c r="D34" s="7">
+        <v>21.0</v>
+      </c>
+      <c r="E34" s="7"/>
+      <c r="F34" s="7">
+        <v>18.0</v>
+      </c>
+      <c r="G34" s="7"/>
+      <c r="H34" s="8"/>
+      <c r="I34" s="8"/>
+      <c r="J34" s="8"/>
+      <c r="K34" s="8"/>
+      <c r="L34" s="8"/>
+    </row>
+    <row r="35" ht="22.5" customHeight="1">
+      <c r="A35" s="6">
+        <v>46171.44421296296</v>
+      </c>
+      <c r="B35" s="6">
+        <v>46171.80347222222</v>
+      </c>
+      <c r="C35" s="7">
+        <v>20.0</v>
+      </c>
+      <c r="D35" s="7">
+        <v>10.0</v>
+      </c>
+      <c r="E35" s="7"/>
+      <c r="F35" s="7">
+        <v>9.0</v>
+      </c>
+      <c r="G35" s="7"/>
+      <c r="H35" s="8"/>
+      <c r="I35" s="8"/>
+      <c r="J35" s="8"/>
+      <c r="K35" s="8"/>
+      <c r="L35" s="8"/>
+    </row>
+    <row r="36" ht="22.5" customHeight="1">
+      <c r="A36" s="6">
+        <v>46170.62986111111</v>
+      </c>
+      <c r="B36" s="6">
+        <v>46171.45570601852</v>
+      </c>
+      <c r="C36" s="7">
+        <v>14.0</v>
+      </c>
+      <c r="D36" s="7">
+        <v>10.0</v>
+      </c>
+      <c r="E36" s="7"/>
+      <c r="F36" s="7"/>
+      <c r="G36" s="7">
+        <v>5.0</v>
+      </c>
+      <c r="H36" s="8"/>
+      <c r="I36" s="8"/>
+      <c r="J36" s="7">
+        <v>18.0</v>
+      </c>
+      <c r="K36" s="8"/>
+      <c r="L36" s="8"/>
+    </row>
+    <row r="37" ht="22.5" customHeight="1">
+      <c r="A37" s="6">
+        <v>46171.45570601852</v>
+      </c>
+      <c r="B37" s="6">
+        <v>46171.80347222222</v>
+      </c>
+      <c r="C37" s="7">
+        <v>16.0</v>
+      </c>
+      <c r="D37" s="7">
+        <v>12.0</v>
+      </c>
+      <c r="E37" s="7"/>
+      <c r="F37" s="7"/>
+      <c r="G37" s="7">
+        <v>6.0</v>
+      </c>
+      <c r="H37" s="8"/>
+      <c r="I37" s="8"/>
+      <c r="J37" s="7"/>
+      <c r="K37" s="8"/>
+      <c r="L37" s="8"/>
+    </row>
+    <row r="38" ht="22.5" customHeight="1">
+      <c r="A38" s="6">
+        <v>46171.51210648148</v>
+      </c>
+      <c r="B38" s="6">
+        <v>46171.80347222222</v>
+      </c>
+      <c r="C38" s="7">
+        <v>11.0</v>
+      </c>
+      <c r="D38" s="7">
+        <v>5.0</v>
+      </c>
+      <c r="E38" s="7"/>
+      <c r="F38" s="7">
+        <v>5.0</v>
+      </c>
+      <c r="G38" s="7"/>
+      <c r="H38" s="8"/>
+      <c r="I38" s="8"/>
+      <c r="J38" s="7"/>
+      <c r="K38" s="8"/>
+      <c r="L38" s="8"/>
+    </row>
+    <row r="39" ht="22.5" customHeight="1">
+      <c r="A39" s="6">
+        <v>46170.63263888889</v>
+      </c>
+      <c r="B39" s="6">
+        <v>46171.43646990741</v>
+      </c>
+      <c r="C39" s="7"/>
+      <c r="D39" s="7">
+        <v>3.0</v>
+      </c>
+      <c r="E39" s="7"/>
+      <c r="F39" s="7"/>
+      <c r="G39" s="7">
+        <v>9.0</v>
+      </c>
+      <c r="H39" s="8"/>
+      <c r="I39" s="8"/>
+      <c r="J39" s="7"/>
+      <c r="K39" s="8"/>
+      <c r="L39" s="8"/>
+    </row>
+    <row r="40" ht="22.5" customHeight="1">
+      <c r="A40" s="6">
+        <v>46171.51416666667</v>
+      </c>
+      <c r="B40" s="6">
+        <v>46171.80347222222</v>
+      </c>
+      <c r="C40" s="7">
+        <v>16.0</v>
+      </c>
+      <c r="D40" s="7">
+        <v>12.0</v>
+      </c>
+      <c r="E40" s="7"/>
+      <c r="F40" s="7"/>
+      <c r="G40" s="7">
+        <v>4.0</v>
+      </c>
+      <c r="H40" s="8"/>
+      <c r="I40" s="8"/>
+      <c r="J40" s="7"/>
+      <c r="K40" s="8"/>
+      <c r="L40" s="8"/>
     </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="A3:B23">
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="A3:B40">
       <formula1>OR(TIMEVALUE(TEXT(A3, "hh:mm:ss"))=A3, AND(ISNUMBER(A3), LEFT(CELL("format", A3))="D"))</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>